<commit_message>
eSpark BOM Template modified
</commit_message>
<xml_diff>
--- a/BOM Format/BOM Template/eSpark.Bom.Template.xlsx
+++ b/BOM Format/BOM Template/eSpark.Bom.Template.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\eSpark-Hardware\BOM Format\BOM Template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\eSpark-Hardware\BOM Format\BOM Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD14786-97DB-4ECA-9AA0-579776306EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Component list</t>
   </si>
@@ -86,21 +85,9 @@
     <t>Column=Comment</t>
   </si>
   <si>
-    <t>Column=Quantity/5 Boards</t>
-  </si>
-  <si>
-    <t>Column=LCSC/MOQ/5 Boards</t>
-  </si>
-  <si>
     <t>Column=Links</t>
   </si>
   <si>
-    <t>Column=Unit Cost/5 Boards</t>
-  </si>
-  <si>
-    <t>Column=Total Cost/5 Boards</t>
-  </si>
-  <si>
     <t>Column=Remarks</t>
   </si>
   <si>
@@ -114,12 +101,24 @@
   </si>
   <si>
     <t>Column=LCSC/Part Number</t>
+  </si>
+  <si>
+    <t>Column=Quantity (5 Boards)</t>
+  </si>
+  <si>
+    <t>Column=MOQ (5 Boards)</t>
+  </si>
+  <si>
+    <t>Column=Total Cost (5 Boards)</t>
+  </si>
+  <si>
+    <t>Column=Unit Cost (5 Boards)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -755,13 +754,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>10417</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>1724025</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
@@ -771,7 +770,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1067,9 +1066,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:T14"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="29" customWidth="1"/>
@@ -1078,21 +1077,21 @@
     <col min="5" max="5" width="30.85546875" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.42578125" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.42578125" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.42578125" customWidth="1"/>
-    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
@@ -1111,10 +1110,9 @@
       <c r="P1" s="62"/>
       <c r="Q1" s="62"/>
       <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="63"/>
+      <c r="S1" s="63"/>
     </row>
-    <row r="2" spans="1:20" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="24"/>
       <c r="C2" s="42"/>
@@ -1126,8 +1124,8 @@
         <v>1</v>
       </c>
       <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1137,10 +1135,9 @@
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="3"/>
+      <c r="S2" s="3"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="25"/>
       <c r="C3" s="43"/>
@@ -1152,8 +1149,8 @@
         <v>3</v>
       </c>
       <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
@@ -1163,10 +1160,9 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="64"/>
+      <c r="S3" s="64"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="25"/>
       <c r="C4" s="43"/>
@@ -1178,8 +1174,8 @@
         <v>5</v>
       </c>
       <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="16"/>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="6"/>
@@ -1189,10 +1185,9 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="65"/>
+      <c r="S4" s="65"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="25"/>
       <c r="C5" s="43"/>
@@ -1204,8 +1199,8 @@
         <v>7</v>
       </c>
       <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="18"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
@@ -1215,10 +1210,9 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="65"/>
+      <c r="S5" s="65"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="26"/>
       <c r="C6" s="44"/>
@@ -1226,8 +1220,8 @@
       <c r="E6" s="19"/>
       <c r="F6" s="20"/>
       <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="18"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
@@ -1237,10 +1231,9 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="65"/>
+      <c r="S6" s="65"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="27"/>
       <c r="C7" s="45"/>
@@ -1248,8 +1241,8 @@
       <c r="E7" s="21"/>
       <c r="F7" s="22"/>
       <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="21"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
@@ -1259,10 +1252,9 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="65"/>
+      <c r="S7" s="65"/>
     </row>
-    <row r="8" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="30"/>
       <c r="C8" s="46"/>
@@ -1270,8 +1262,8 @@
       <c r="E8" s="31"/>
       <c r="F8" s="32"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="21"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
@@ -1281,16 +1273,15 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="65"/>
+      <c r="S8" s="65"/>
     </row>
-    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="33" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>13</v>
@@ -1305,13 +1296,13 @@
         <v>15</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I9" s="33" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J9" s="33" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K9" s="33" t="s">
         <v>17</v>
@@ -1320,31 +1311,28 @@
         <v>10</v>
       </c>
       <c r="M9" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="N9" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="O9" s="33" t="s">
+      <c r="P9" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q9" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="R9" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="P9" s="33" t="s">
+      <c r="S9" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="Q9" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="R9" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="S9" s="35" t="s">
-        <v>23</v>
-      </c>
-      <c r="T9" s="35" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="10" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="41">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1365,11 +1353,10 @@
       <c r="O10" s="50"/>
       <c r="P10" s="50"/>
       <c r="Q10" s="50"/>
-      <c r="R10" s="50"/>
-      <c r="S10" s="52"/>
-      <c r="T10" s="53"/>
+      <c r="R10" s="52"/>
+      <c r="S10" s="53"/>
     </row>
-    <row r="11" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="41">
         <f t="shared" ref="B11:B12" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1390,11 +1377,10 @@
       <c r="O11" s="54"/>
       <c r="P11" s="54"/>
       <c r="Q11" s="54"/>
-      <c r="R11" s="54"/>
-      <c r="S11" s="56"/>
-      <c r="T11" s="57"/>
+      <c r="R11" s="56"/>
+      <c r="S11" s="57"/>
     </row>
-    <row r="12" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="41">
         <f t="shared" si="0"/>
@@ -1415,11 +1401,10 @@
       <c r="O12" s="58"/>
       <c r="P12" s="58"/>
       <c r="Q12" s="58"/>
-      <c r="R12" s="58"/>
-      <c r="S12" s="60"/>
-      <c r="T12" s="61"/>
+      <c r="R12" s="60"/>
+      <c r="S12" s="61"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="36"/>
       <c r="C13" s="48"/>
@@ -1429,8 +1414,8 @@
       <c r="E13" s="38"/>
       <c r="F13" s="39"/>
       <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="40"/>
       <c r="J13" s="39"/>
       <c r="K13" s="40"/>
       <c r="L13" s="40"/>
@@ -1439,11 +1424,10 @@
       <c r="O13" s="40"/>
       <c r="P13" s="40"/>
       <c r="Q13" s="40"/>
-      <c r="R13" s="40"/>
-      <c r="S13" s="66"/>
-      <c r="T13" s="67"/>
+      <c r="R13" s="66"/>
+      <c r="S13" s="67"/>
     </row>
-    <row r="14" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="28"/>
       <c r="C14" s="49"/>
@@ -1463,15 +1447,14 @@
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
       <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="68"/>
-      <c r="T14" s="69"/>
+      <c r="R14" s="68"/>
+      <c r="S14" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="K1:T1"/>
-    <mergeCell ref="T3:T8"/>
-    <mergeCell ref="S13:T14"/>
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="R13:S14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>